<commit_message>
Add real-name completion duration event
</commit_message>
<xml_diff>
--- a/编辑中-采集方案-账号中心.xlsx
+++ b/编辑中-采集方案-账号中心.xlsx
@@ -3900,7 +3900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J90"/>
+  <dimension ref="A1:J94"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.3846153846154" defaultRowHeight="17.6"/>
   <cols>
     <col width="14.4230769230769" customWidth="1" style="80" min="1" max="1"/>
@@ -6526,10 +6526,124 @@
       <c r="I90" s="108" t="n"/>
       <c r="J90" s="132" t="n"/>
     </row>
-    <row r="91" ht="18" customFormat="1" customHeight="1" s="79"/>
-    <row r="92" ht="18" customFormat="1" customHeight="1" s="79"/>
-    <row r="93" ht="18" customFormat="1" customHeight="1" s="79"/>
-    <row r="94" ht="18" customFormat="1" customHeight="1" s="79"/>
+    <row r="91" ht="18" customFormat="1" customHeight="1" s="79">
+      <c r="A91" s="153" t="n">
+        <v>20</v>
+      </c>
+      <c r="B91" s="109" t="inlineStr">
+        <is>
+          <t>realname_complete_time</t>
+        </is>
+      </c>
+      <c r="C91" s="109" t="inlineStr">
+        <is>
+          <t>实名认证_提交到完成时长</t>
+        </is>
+      </c>
+      <c r="D91" s="106" t="n"/>
+      <c r="E91" s="109" t="inlineStr">
+        <is>
+          <t>$预置属性</t>
+        </is>
+      </c>
+      <c r="F91" s="106" t="n"/>
+      <c r="G91" s="125" t="n"/>
+      <c r="H91" s="153" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="I91" s="109" t="inlineStr">
+        <is>
+          <t>认证最终完成时触发，覆盖提交到完成的时长</t>
+        </is>
+      </c>
+      <c r="J91" s="132" t="n"/>
+    </row>
+    <row r="92" ht="18" customFormat="1" customHeight="1" s="79">
+      <c r="A92" s="107" t="n"/>
+      <c r="B92" s="108" t="n"/>
+      <c r="C92" s="108" t="n"/>
+      <c r="D92" s="109" t="inlineStr">
+        <is>
+          <t>page_name</t>
+        </is>
+      </c>
+      <c r="E92" s="109" t="inlineStr">
+        <is>
+          <t>页面名称</t>
+        </is>
+      </c>
+      <c r="F92" s="109" t="inlineStr">
+        <is>
+          <t>STRING</t>
+        </is>
+      </c>
+      <c r="G92" s="127" t="inlineStr">
+        <is>
+          <t>实名认证提交成功页、实名认证审核中页</t>
+        </is>
+      </c>
+      <c r="H92" s="107" t="n"/>
+      <c r="I92" s="108" t="n"/>
+      <c r="J92" s="132" t="n"/>
+    </row>
+    <row r="93" ht="18" customFormat="1" customHeight="1" s="79">
+      <c r="A93" s="107" t="n"/>
+      <c r="B93" s="108" t="n"/>
+      <c r="C93" s="108" t="n"/>
+      <c r="D93" s="109" t="inlineStr">
+        <is>
+          <t>attestation_type</t>
+        </is>
+      </c>
+      <c r="E93" s="109" t="inlineStr">
+        <is>
+          <t>认证方式</t>
+        </is>
+      </c>
+      <c r="F93" s="109" t="inlineStr">
+        <is>
+          <t>STRING</t>
+        </is>
+      </c>
+      <c r="G93" s="127" t="inlineStr">
+        <is>
+          <t>个人认证、企业认证</t>
+        </is>
+      </c>
+      <c r="H93" s="107" t="n"/>
+      <c r="I93" s="108" t="n"/>
+      <c r="J93" s="132" t="n"/>
+    </row>
+    <row r="94" ht="18" customFormat="1" customHeight="1" s="79">
+      <c r="A94" s="107" t="n"/>
+      <c r="B94" s="108" t="n"/>
+      <c r="C94" s="108" t="n"/>
+      <c r="D94" s="109" t="inlineStr">
+        <is>
+          <t>duration</t>
+        </is>
+      </c>
+      <c r="E94" s="109" t="inlineStr">
+        <is>
+          <t>耗时</t>
+        </is>
+      </c>
+      <c r="F94" s="109" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="G94" s="127" t="inlineStr">
+        <is>
+          <t>从提交成功到认证状态完成的时长，单位按研发口径上报，单位：毫秒</t>
+        </is>
+      </c>
+      <c r="H94" s="107" t="n"/>
+      <c r="I94" s="108" t="n"/>
+      <c r="J94" s="132" t="n"/>
+    </row>
     <row r="95" ht="18" customFormat="1" customHeight="1" s="79"/>
     <row r="96" ht="18" customFormat="1" customHeight="1" s="79"/>
     <row r="97" ht="18" customFormat="1" customHeight="1" s="79"/>
@@ -13463,9 +13577,9 @@
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="A13:A23"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A26:A36"/>
     <mergeCell ref="A46:O47"/>
-    <mergeCell ref="A26:A36"/>
-    <mergeCell ref="A24:A25"/>
     <mergeCell ref="A69:N69"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="C79:E79"/>

</xml_diff>